<commit_message>
Juno: check in to OLPRODLOC.
</commit_message>
<xml_diff>
--- a/ResourceFiles/Contoso Chai Tea market trends 2023.xlsx
+++ b/ResourceFiles/Contoso Chai Tea market trends 2023.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <r>
       <rPr>
@@ -117,7 +117,18 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>4:36</t>
+      <t>3:15</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>5:48</t>
     </r>
   </si>
   <si>
@@ -867,11 +878,11 @@
       <c r="C6">
         <v>499</v>
       </c>
-      <c r="D6" t="s">
-        <v>6</v>
+      <c r="D6">
+        <v>436</v>
       </c>
       <c r="E6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6">
         <v>2996</v>
@@ -885,11 +896,11 @@
         <f t="shared" si="0"/>
         <v>863</v>
       </c>
-      <c r="C7">
-        <v>315</v>
-      </c>
-      <c r="D7">
-        <v>548</v>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
       </c>
       <c r="E7">
         <v>3599</v>

</xml_diff>

<commit_message>
Copy Files From Source Repo (2025-10-11 14:36)
</commit_message>
<xml_diff>
--- a/ResourceFiles/Contoso Chai Tea market trends 2023.xlsx
+++ b/ResourceFiles/Contoso Chai Tea market trends 2023.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <r>
       <rPr>
@@ -117,7 +117,18 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>4:36</t>
+      <t>3:15</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>5:48</t>
     </r>
   </si>
   <si>
@@ -867,11 +878,11 @@
       <c r="C6">
         <v>499</v>
       </c>
-      <c r="D6" t="s">
-        <v>6</v>
+      <c r="D6">
+        <v>436</v>
       </c>
       <c r="E6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6">
         <v>2996</v>
@@ -885,11 +896,11 @@
         <f t="shared" si="0"/>
         <v>863</v>
       </c>
-      <c r="C7">
-        <v>315</v>
-      </c>
-      <c r="D7">
-        <v>548</v>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
       </c>
       <c r="E7">
         <v>3599</v>

</xml_diff>